<commit_message>
Record executed results for 30 black-box cases with reports and evidence
</commit_message>
<xml_diff>
--- a/TEST_CASE_HOP_DEN.xlsx
+++ b/TEST_CASE_HOP_DEN.xlsx
@@ -525,7 +525,7 @@
       <c r="E2" s="2" t="inlineStr">
         <is>
           <t>1. Bấm Đăng ký độc giả.
-2. Nhập dữ liệu trên, bấm Đăng ký.
+2. Nhập dữ liệu trên, bấm Tạo tài khoản.
 3. Đăng nhập tài khoản vừa tạo.</t>
         </is>
       </c>
@@ -571,7 +571,7 @@
         <is>
           <t>1. Mở Đăng ký độc giả.
 2. Điền họ tên/mật khẩu, để trống tên đăng nhập.
-3. Bấm Đăng ký.</t>
+3. Bấm Tạo tài khoản.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -612,7 +612,7 @@
         <is>
           <t>1. Mở Đăng ký độc giả.
 2. Dùng username readerRUN, họ tên/mật khẩu hợp lệ.
-3. Bấm Đăng ký.</t>
+3. Bấm Tạo tài khoản.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">

</xml_diff>